<commit_message>
NAKO-DPE AND DD From Tracy,Ines and Franzi
</commit_message>
<xml_diff>
--- a/analyst/Franzi/rmonize/data_dictionary/DD_NAKO_FRANZI.xlsx
+++ b/analyst/Franzi/rmonize/data_dictionary/DD_NAKO_FRANZI.xlsx
@@ -1,22 +1,129 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\use-cases-harmonisation\use-cases-harmonisation\analyst\Franzi\rmonize\data_dictionary\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD669241-6B49-41F0-AAAA-338AF752B63B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" r:id="rId1"/>
     <sheet name="Categories" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="32">
+  <si>
+    <t>index</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>label</t>
+  </si>
+  <si>
+    <t>valueType</t>
+  </si>
+  <si>
+    <t>variable</t>
+  </si>
+  <si>
+    <t>a_ui_m11</t>
+  </si>
+  <si>
+    <t>main group sugar, sweets[g/d]</t>
+  </si>
+  <si>
+    <t>decimal</t>
+  </si>
+  <si>
+    <t>a_ui_m12</t>
+  </si>
+  <si>
+    <t>Main group cake[g/d]</t>
+  </si>
+  <si>
+    <t>a_ui_f1301</t>
+  </si>
+  <si>
+    <t>Fruit and vegetable juices[g/d]</t>
+  </si>
+  <si>
+    <t>a_ui_f1302</t>
+  </si>
+  <si>
+    <t>Soft drinks[g/d]</t>
+  </si>
+  <si>
+    <t>a_ui_m02</t>
+  </si>
+  <si>
+    <t>Main group vegetables[g/d]</t>
+  </si>
+  <si>
+    <t>a_ui_m03</t>
+  </si>
+  <si>
+    <t>Main group pulses[g/d]</t>
+  </si>
+  <si>
+    <t>a_ui_f0401</t>
+  </si>
+  <si>
+    <t>Fruits[g/d]</t>
+  </si>
+  <si>
+    <t>a_ui_f070100</t>
+  </si>
+  <si>
+    <t>Fresh meat unclassified[g/d]</t>
+  </si>
+  <si>
+    <t>a_ui_f070101</t>
+  </si>
+  <si>
+    <t>Beef[g/d]</t>
+  </si>
+  <si>
+    <t>a_ui_f070103</t>
+  </si>
+  <si>
+    <t>Pork[g/d]</t>
+  </si>
+  <si>
+    <t>a_ui_f0704</t>
+  </si>
+  <si>
+    <t>a_ui_f130301</t>
+  </si>
+  <si>
+    <t>Coffee[g/d]</t>
+  </si>
+  <si>
+    <t>a_ui_f130302</t>
+  </si>
+  <si>
+    <t>Tea[g/d]</t>
+  </si>
+  <si>
+    <t>process meat[g/d]</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -28,6 +135,19 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -53,10 +173,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -64,6 +191,14 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -110,7 +245,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -142,9 +277,27 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -176,6 +329,24 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -351,31 +522,174 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>index</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>label</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>valueType</t>
-        </is>
-      </c>
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="B2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="B6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B8" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B9" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B10" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B11" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B12" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B13" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B14" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B16" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -383,25 +697,19 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>variable</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>label</t>
-        </is>
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
NAKO-FOOD ITEMS we need total fruits intake not fresh fruits intake. This has been corrected now.
</commit_message>
<xml_diff>
--- a/analyst/Franzi/rmonize/data_dictionary/DD_NAKO_FRANZI.xlsx
+++ b/analyst/Franzi/rmonize/data_dictionary/DD_NAKO_FRANZI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\use-cases-harmonisation\use-cases-harmonisation\analyst\Franzi\rmonize\data_dictionary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD42BCED-2B8A-4BDC-8D68-E69A6319EBC0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E76D5EA5-CB56-497C-893B-C88077883034}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -77,12 +77,6 @@
     <t>Main group pulses[g/d]</t>
   </si>
   <si>
-    <t>a_ui_f0401</t>
-  </si>
-  <si>
-    <t>Fruits[g/d]</t>
-  </si>
-  <si>
     <t>a_ui_f070100</t>
   </si>
   <si>
@@ -117,6 +111,12 @@
   </si>
   <si>
     <t>process meat[g/d]</t>
+  </si>
+  <si>
+    <t>a_ui_m04</t>
+  </si>
+  <si>
+    <t>Main group Fruits, nuts[g/d]</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
@@ -648,8 +648,8 @@
       <c r="B11" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>25</v>
+      <c r="C11" s="2" t="s">
+        <v>29</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>7</v>
@@ -657,10 +657,10 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B12" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>26</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>31</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>7</v>
@@ -679,17 +679,17 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B14" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B16" s="3"/>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B15" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>